<commit_message>
fix: promote verified digital product xlsx assets
</commit_message>
<xml_diff>
--- a/digital-products/hdb-renosmart-planner/HDB-RenoSmart-Budget-Compliance-Planner-2026.xlsx
+++ b/digital-products/hdb-renosmart-planner/HDB-RenoSmart-Budget-Compliance-Planner-2026.xlsx
@@ -38,8 +38,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="&quot;S$&quot;#,##0"/>
+    <numFmt numFmtId="61" formatCode="0.0%"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -70,8 +72,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="61" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -570,10 +574,10 @@
       <c r="B7" t="str">
         <v>kitchen</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <v>8900</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="1">
         <v>23200</v>
       </c>
       <c r="E7" t="str">
@@ -587,10 +591,10 @@
       <c r="B8" t="str">
         <v>bathroom</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>2600</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="1">
         <v>5200</v>
       </c>
       <c r="E8" t="str">
@@ -604,10 +608,10 @@
       <c r="B9" t="str">
         <v>flooring</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <v>5000</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="1">
         <v>12000</v>
       </c>
       <c r="E9" t="str">
@@ -621,10 +625,10 @@
       <c r="B10" t="str">
         <v>painting</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>2500</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="1">
         <v>6000</v>
       </c>
       <c r="E10" t="str">
@@ -638,10 +642,10 @@
       <c r="B11" t="str">
         <v>carpentry</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>6000</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="1">
         <v>15000</v>
       </c>
       <c r="E11" t="str">
@@ -655,10 +659,10 @@
       <c r="B12" t="str">
         <v>electrical</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <v>3000</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="1">
         <v>6000</v>
       </c>
       <c r="E12" t="str">
@@ -672,10 +676,10 @@
       <c r="B13" t="str">
         <v>hacking</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <v>2000</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <v>6000</v>
       </c>
       <c r="E13" t="str">
@@ -689,10 +693,10 @@
       <c r="B14" t="str">
         <v>builtin</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <v>6000</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="1">
         <v>15000</v>
       </c>
       <c r="E14" t="str">
@@ -706,10 +710,10 @@
       <c r="B15" t="str">
         <v>appliances</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <v>3000</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="1">
         <v>10000</v>
       </c>
       <c r="E15" t="str">
@@ -723,10 +727,10 @@
       <c r="B16" t="str">
         <v>userdefined</v>
       </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
+      <c r="C16" s="1">
+        <v>0</v>
+      </c>
+      <c r="D16" s="1">
         <v>0</v>
       </c>
       <c r="E16" t="str">
@@ -908,7 +912,7 @@
       <c r="B39" t="str">
         <v>Light</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="2">
         <v>0.08</v>
       </c>
       <c r="D39" t="str">
@@ -922,7 +926,7 @@
       <c r="B40" t="str">
         <v>Moderate</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="2">
         <v>0.12</v>
       </c>
       <c r="D40" t="str">
@@ -936,7 +940,7 @@
       <c r="B41" t="str">
         <v>Extensive</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="2">
         <v>0.15</v>
       </c>
       <c r="D41" t="str">
@@ -955,7 +959,7 @@
       <c r="B44" t="str">
         <v>Current GST rate</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="2">
         <v>0.09</v>
       </c>
       <c r="D44" t="str">
@@ -1004,7 +1008,7 @@
       <c r="B51" t="str">
         <v>Deposit at signing</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="2">
         <v>0.15</v>
       </c>
       <c r="D51" t="str">
@@ -1015,7 +1019,7 @@
       <c r="B52" t="str">
         <v>Hacking / demolition complete</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="2">
         <v>0.2</v>
       </c>
       <c r="D52" t="str">
@@ -1026,7 +1030,7 @@
       <c r="B53" t="str">
         <v>Wet works complete (tiling, waterproofing)</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="2">
         <v>0.3</v>
       </c>
       <c r="D53" t="str">
@@ -1037,7 +1041,7 @@
       <c r="B54" t="str">
         <v>Carpentry &amp; M&amp;E complete</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="2">
         <v>0.2</v>
       </c>
       <c r="D54" t="str">
@@ -1048,7 +1052,7 @@
       <c r="B55" t="str">
         <v>Final on completion</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="2">
         <v>0.15</v>
       </c>
       <c r="D55" t="str">
@@ -1059,7 +1063,7 @@
       <c r="B56" t="str">
         <v>Total (must = 100%)</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="2">
         <f>SUM(C51:C55)</f>
         <v>0</v>
       </c>
@@ -1119,7 +1123,7 @@
       <c r="B8" t="str">
         <v>Floor area (sqm)</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>90</v>
       </c>
       <c r="D8" t="str">
@@ -1163,22 +1167,22 @@
       <c r="B13" t="str">
         <v>Kitchen renovation</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <f>ROUND(ASSUMPTIONS!C7*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <f>ROUND(ASSUMPTIONS!D7*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E13" s="1" t="str">
         <v/>
       </c>
-      <c r="F13">
+      <c r="F13" s="1">
         <f>IF($E13="",C13,$E13)</f>
         <v>0</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="1">
         <f>IF($E13="",D13,$E13)</f>
         <v>0</v>
       </c>
@@ -1187,22 +1191,22 @@
       <c r="B14" t="str">
         <v>Bathroom renovation</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <f>ROUND(ASSUMPTIONS!C8*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="1">
         <f>ROUND(ASSUMPTIONS!D8*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E14" s="1" t="str">
         <v/>
       </c>
-      <c r="F14">
+      <c r="F14" s="1">
         <f>IF($E14="",C14,$E14)</f>
         <v>0</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <f>IF($E14="",D14,$E14)</f>
         <v>0</v>
       </c>
@@ -1211,22 +1215,22 @@
       <c r="B15" t="str">
         <v>Flooring</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <f>ROUND(ASSUMPTIONS!C9*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="1">
         <f>ROUND(ASSUMPTIONS!D9*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E15" s="1" t="str">
         <v/>
       </c>
-      <c r="F15">
+      <c r="F15" s="1">
         <f>IF($E15="",C15,$E15)</f>
         <v>0</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="1">
         <f>IF($E15="",D15,$E15)</f>
         <v>0</v>
       </c>
@@ -1235,22 +1239,22 @@
       <c r="B16" t="str">
         <v>Painting</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <f>ROUND(ASSUMPTIONS!C10*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="1">
         <f>ROUND(ASSUMPTIONS!D10*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E16" t="str">
+      <c r="E16" s="1" t="str">
         <v/>
       </c>
-      <c r="F16">
+      <c r="F16" s="1">
         <f>IF($E16="",C16,$E16)</f>
         <v>0</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="1">
         <f>IF($E16="",D16,$E16)</f>
         <v>0</v>
       </c>
@@ -1259,22 +1263,22 @@
       <c r="B17" t="str">
         <v>Carpentry</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="1">
         <f>ROUND(ASSUMPTIONS!C11*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="1">
         <f>ROUND(ASSUMPTIONS!D11*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E17" t="str">
+      <c r="E17" s="1" t="str">
         <v/>
       </c>
-      <c r="F17">
+      <c r="F17" s="1">
         <f>IF($E17="",C17,$E17)</f>
         <v>0</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <f>IF($E17="",D17,$E17)</f>
         <v>0</v>
       </c>
@@ -1283,22 +1287,22 @@
       <c r="B18" t="str">
         <v>Electrical</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="1">
         <f>ROUND(ASSUMPTIONS!C12*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="1">
         <f>ROUND(ASSUMPTIONS!D12*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E18" t="str">
+      <c r="E18" s="1" t="str">
         <v/>
       </c>
-      <c r="F18">
+      <c r="F18" s="1">
         <f>IF($E18="",C18,$E18)</f>
         <v>0</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="1">
         <f>IF($E18="",D18,$E18)</f>
         <v>0</v>
       </c>
@@ -1307,22 +1311,22 @@
       <c r="B19" t="str">
         <v>Hacking</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <f>ROUND(ASSUMPTIONS!C13*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="1">
         <f>ROUND(ASSUMPTIONS!D13*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E19" t="str">
+      <c r="E19" s="1" t="str">
         <v/>
       </c>
-      <c r="F19">
+      <c r="F19" s="1">
         <f>IF($E19="",C19,$E19)</f>
         <v>0</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="1">
         <f>IF($E19="",D19,$E19)</f>
         <v>0</v>
       </c>
@@ -1331,22 +1335,22 @@
       <c r="B20" t="str">
         <v>Built-in furniture</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <f>ROUND(ASSUMPTIONS!C14*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="1">
         <f>ROUND(ASSUMPTIONS!D14*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E20" t="str">
+      <c r="E20" s="1" t="str">
         <v/>
       </c>
-      <c r="F20">
+      <c r="F20" s="1">
         <f>IF($E20="",C20,$E20)</f>
         <v>0</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="1">
         <f>IF($E20="",D20,$E20)</f>
         <v>0</v>
       </c>
@@ -1355,22 +1359,22 @@
       <c r="B21" t="str">
         <v>Appliances / optional items</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="1">
         <f>ROUND(ASSUMPTIONS!C15*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="1">
         <f>ROUND(ASSUMPTIONS!D15*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E21" s="1" t="str">
         <v/>
       </c>
-      <c r="F21">
+      <c r="F21" s="1">
         <f>IF($E21="",C21,$E21)</f>
         <v>0</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="1">
         <f>IF($E21="",D21,$E21)</f>
         <v>0</v>
       </c>
@@ -1379,22 +1383,22 @@
       <c r="B22" t="str">
         <v>User-defined costs</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <f>ROUND(ASSUMPTIONS!C16*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="1">
         <f>ROUND(ASSUMPTIONS!D16*(IF($C$7="BTO",ASSUMPTIONS!C20,ASSUMPTIONS!C21))*(IF($C$9="Light",ASSUMPTIONS!C25,IF($C$9="Extensive",ASSUMPTIONS!C27,ASSUMPTIONS!C26)))*(IF(ASSUMPTIONS!C35=1.0,ROUND(($C$8/90)^0.6,3),ASSUMPTIONS!C35)),0)</f>
         <v>0</v>
       </c>
-      <c r="E22" t="str">
+      <c r="E22" s="1" t="str">
         <v/>
       </c>
-      <c r="F22">
+      <c r="F22" s="1">
         <f>IF($E22="",C22,$E22)</f>
         <v>0</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="1">
         <f>IF($E22="",D22,$E22)</f>
         <v>0</v>
       </c>
@@ -1403,7 +1407,7 @@
       <c r="B24" t="str">
         <v>ESTIMATED BASE BUDGET (mid-point of auto/quotes)</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="1">
         <f>(SUM(F13:F22)+SUM(G13:G22))/2</f>
         <v>0</v>
       </c>
@@ -1412,7 +1416,7 @@
       <c r="B25" t="str">
         <v>LOW PLANNING RANGE</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="1">
         <f>SUM(F13:F22)</f>
         <v>0</v>
       </c>
@@ -1421,7 +1425,7 @@
       <c r="B26" t="str">
         <v>HIGH PLANNING RANGE</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="1">
         <f>SUM(G13:G22)</f>
         <v>0</v>
       </c>
@@ -1433,7 +1437,7 @@
       <c r="D27" t="str">
         <v>Assumes baseline prices are GST-exclusive. Set ASSUMPTIONS!C45 to TRUE if quotes include GST</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="1">
         <f>IF(ASSUMPTIONS!C45,0,ROUND(F24*ASSUMPTIONS!C44,0))</f>
         <v>0</v>
       </c>
@@ -1447,7 +1451,7 @@
       <c r="B29" t="str">
         <v>Contingency rate</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="2">
         <f>IF($C$9="Light",ASSUMPTIONS!C39,IF($C$9="Extensive",ASSUMPTIONS!C41,ASSUMPTIONS!C40))</f>
         <v>0</v>
       </c>
@@ -1459,7 +1463,7 @@
       <c r="B30" t="str">
         <v>Optional items subtotal (appliances + user-defined)</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <f>(F21+G21+F22+G22)/2</f>
         <v>0</v>
       </c>
@@ -1468,7 +1472,7 @@
       <c r="B31" t="str">
         <v>ESTIMATED TOTAL (base + GST + contingency)</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <f>ROUND(F24+F27+F24*C29,0)</f>
         <v>0</v>
       </c>
@@ -1482,7 +1486,7 @@
       <c r="B34" t="str">
         <v>Renovation loan planned (S$)</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="1">
         <v>0</v>
       </c>
     </row>
@@ -1490,7 +1494,7 @@
       <c r="B35" t="str">
         <v>Contingency reserve amount</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="1">
         <f>ROUND(F24*C29,0)</f>
         <v>0</v>
       </c>
@@ -1499,7 +1503,7 @@
       <c r="B36" t="str">
         <v>CASH YOU MUST COVER (total − loan)</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="1">
         <f>MAX(0,E31-C34)</f>
         <v>0</v>
       </c>
@@ -1528,11 +1532,11 @@
         <f>ASSUMPTIONS!B51</f>
         <v>0</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="2">
         <f>ASSUMPTIONS!C51</f>
         <v>0</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="1">
         <f>ROUND(E31*C40,0)</f>
         <v>0</v>
       </c>
@@ -1546,11 +1550,11 @@
         <f>ASSUMPTIONS!B52</f>
         <v>0</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="2">
         <f>ASSUMPTIONS!C52</f>
         <v>0</v>
       </c>
-      <c r="D41">
+      <c r="D41" s="1">
         <f>ROUND(E31*C41,0)</f>
         <v>0</v>
       </c>
@@ -1564,11 +1568,11 @@
         <f>ASSUMPTIONS!B53</f>
         <v>0</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="2">
         <f>ASSUMPTIONS!C53</f>
         <v>0</v>
       </c>
-      <c r="D42">
+      <c r="D42" s="1">
         <f>ROUND(E31*C42,0)</f>
         <v>0</v>
       </c>
@@ -1582,11 +1586,11 @@
         <f>ASSUMPTIONS!B54</f>
         <v>0</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="2">
         <f>ASSUMPTIONS!C54</f>
         <v>0</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="1">
         <f>ROUND(E31*C43,0)</f>
         <v>0</v>
       </c>
@@ -1600,11 +1604,11 @@
         <f>ASSUMPTIONS!B55</f>
         <v>0</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="2">
         <f>ASSUMPTIONS!C55</f>
         <v>0</v>
       </c>
-      <c r="D44">
+      <c r="D44" s="1">
         <f>ROUND(E31*C44,0)</f>
         <v>0</v>
       </c>
@@ -1617,7 +1621,7 @@
       <c r="B45" t="str">
         <v>Total (must = 100%)</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="2">
         <f>SUM(C40:C44)</f>
         <v>0</v>
       </c>
@@ -1760,11 +1764,11 @@
       <c r="B14" t="str">
         <v>Kitchen renovation</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <f>ASSUMPTIONS!C7</f>
         <v>0</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="1">
         <f>ASSUMPTIONS!D7</f>
         <v>0</v>
       </c>
@@ -1772,27 +1776,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="1">
         <f>ROUND(C14*E14,0)</f>
         <v>0</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="1">
         <f>ROUND(D14*E14,0)</f>
         <v>0</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="1">
         <f>INPUTS!E13</f>
         <v>0</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="1">
         <f>INPUTS!E13</f>
         <v>0</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="1">
         <f>IF(H14="",F14,H14)</f>
         <v>0</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="1">
         <f>IF(I14="",G14,I14)</f>
         <v>0</v>
       </c>
@@ -1801,11 +1805,11 @@
       <c r="B15" t="str">
         <v>Bathroom renovation</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <f>ASSUMPTIONS!C8</f>
         <v>0</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="1">
         <f>ASSUMPTIONS!D8</f>
         <v>0</v>
       </c>
@@ -1813,27 +1817,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="1">
         <f>ROUND(C15*E15,0)</f>
         <v>0</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="1">
         <f>ROUND(D15*E15,0)</f>
         <v>0</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="1">
         <f>INPUTS!E14</f>
         <v>0</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="1">
         <f>INPUTS!E14</f>
         <v>0</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="1">
         <f>IF(H15="",F15,H15)</f>
         <v>0</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="1">
         <f>IF(I15="",G15,I15)</f>
         <v>0</v>
       </c>
@@ -1842,11 +1846,11 @@
       <c r="B16" t="str">
         <v>Flooring</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <f>ASSUMPTIONS!C9</f>
         <v>0</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="1">
         <f>ASSUMPTIONS!D9</f>
         <v>0</v>
       </c>
@@ -1854,27 +1858,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="1">
         <f>ROUND(C16*E16,0)</f>
         <v>0</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="1">
         <f>ROUND(D16*E16,0)</f>
         <v>0</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="1">
         <f>INPUTS!E15</f>
         <v>0</v>
       </c>
-      <c r="I16">
+      <c r="I16" s="1">
         <f>INPUTS!E15</f>
         <v>0</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="1">
         <f>IF(H16="",F16,H16)</f>
         <v>0</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="1">
         <f>IF(I16="",G16,I16)</f>
         <v>0</v>
       </c>
@@ -1883,11 +1887,11 @@
       <c r="B17" t="str">
         <v>Painting</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="1">
         <f>ASSUMPTIONS!C10</f>
         <v>0</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="1">
         <f>ASSUMPTIONS!D10</f>
         <v>0</v>
       </c>
@@ -1895,27 +1899,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="1">
         <f>ROUND(C17*E17,0)</f>
         <v>0</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="1">
         <f>ROUND(D17*E17,0)</f>
         <v>0</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="1">
         <f>INPUTS!E16</f>
         <v>0</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="1">
         <f>INPUTS!E16</f>
         <v>0</v>
       </c>
-      <c r="J17">
+      <c r="J17" s="1">
         <f>IF(H17="",F17,H17)</f>
         <v>0</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="1">
         <f>IF(I17="",G17,I17)</f>
         <v>0</v>
       </c>
@@ -1924,11 +1928,11 @@
       <c r="B18" t="str">
         <v>Carpentry</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="1">
         <f>ASSUMPTIONS!C11</f>
         <v>0</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="1">
         <f>ASSUMPTIONS!D11</f>
         <v>0</v>
       </c>
@@ -1936,27 +1940,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="1">
         <f>ROUND(C18*E18,0)</f>
         <v>0</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="1">
         <f>ROUND(D18*E18,0)</f>
         <v>0</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="1">
         <f>INPUTS!E17</f>
         <v>0</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="1">
         <f>INPUTS!E17</f>
         <v>0</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="1">
         <f>IF(H18="",F18,H18)</f>
         <v>0</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="1">
         <f>IF(I18="",G18,I18)</f>
         <v>0</v>
       </c>
@@ -1965,11 +1969,11 @@
       <c r="B19" t="str">
         <v>Electrical</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <f>ASSUMPTIONS!C12</f>
         <v>0</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="1">
         <f>ASSUMPTIONS!D12</f>
         <v>0</v>
       </c>
@@ -1977,27 +1981,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="1">
         <f>ROUND(C19*E19,0)</f>
         <v>0</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="1">
         <f>ROUND(D19*E19,0)</f>
         <v>0</v>
       </c>
-      <c r="H19">
+      <c r="H19" s="1">
         <f>INPUTS!E18</f>
         <v>0</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="1">
         <f>INPUTS!E18</f>
         <v>0</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="1">
         <f>IF(H19="",F19,H19)</f>
         <v>0</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="1">
         <f>IF(I19="",G19,I19)</f>
         <v>0</v>
       </c>
@@ -2006,11 +2010,11 @@
       <c r="B20" t="str">
         <v>Hacking</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <f>ASSUMPTIONS!C13</f>
         <v>0</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="1">
         <f>ASSUMPTIONS!D13</f>
         <v>0</v>
       </c>
@@ -2018,27 +2022,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="1">
         <f>ROUND(C20*E20,0)</f>
         <v>0</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="1">
         <f>ROUND(D20*E20,0)</f>
         <v>0</v>
       </c>
-      <c r="H20">
+      <c r="H20" s="1">
         <f>INPUTS!E19</f>
         <v>0</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="1">
         <f>INPUTS!E19</f>
         <v>0</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="1">
         <f>IF(H20="",F20,H20)</f>
         <v>0</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="1">
         <f>IF(I20="",G20,I20)</f>
         <v>0</v>
       </c>
@@ -2047,11 +2051,11 @@
       <c r="B21" t="str">
         <v>Built-in furniture</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="1">
         <f>ASSUMPTIONS!C14</f>
         <v>0</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="1">
         <f>ASSUMPTIONS!D14</f>
         <v>0</v>
       </c>
@@ -2059,27 +2063,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="1">
         <f>ROUND(C21*E21,0)</f>
         <v>0</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="1">
         <f>ROUND(D21*E21,0)</f>
         <v>0</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="1">
         <f>INPUTS!E20</f>
         <v>0</v>
       </c>
-      <c r="I21">
+      <c r="I21" s="1">
         <f>INPUTS!E20</f>
         <v>0</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="1">
         <f>IF(H21="",F21,H21)</f>
         <v>0</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="1">
         <f>IF(I21="",G21,I21)</f>
         <v>0</v>
       </c>
@@ -2088,11 +2092,11 @@
       <c r="B22" t="str">
         <v>Appliances / optional items</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <f>ASSUMPTIONS!C15</f>
         <v>0</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="1">
         <f>ASSUMPTIONS!D15</f>
         <v>0</v>
       </c>
@@ -2100,27 +2104,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="1">
         <f>ROUND(C22*E22,0)</f>
         <v>0</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="1">
         <f>ROUND(D22*E22,0)</f>
         <v>0</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="1">
         <f>INPUTS!E21</f>
         <v>0</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="1">
         <f>INPUTS!E21</f>
         <v>0</v>
       </c>
-      <c r="J22">
+      <c r="J22" s="1">
         <f>IF(H22="",F22,H22)</f>
         <v>0</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="1">
         <f>IF(I22="",G22,I22)</f>
         <v>0</v>
       </c>
@@ -2129,11 +2133,11 @@
       <c r="B23" t="str">
         <v>User-defined costs</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="1">
         <f>ASSUMPTIONS!C16</f>
         <v>0</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="1">
         <f>ASSUMPTIONS!D16</f>
         <v>0</v>
       </c>
@@ -2141,27 +2145,27 @@
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="1">
         <f>ROUND(C23*E23,0)</f>
         <v>0</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="1">
         <f>ROUND(D23*E23,0)</f>
         <v>0</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="1">
         <f>INPUTS!E22</f>
         <v>0</v>
       </c>
-      <c r="I23">
+      <c r="I23" s="1">
         <f>INPUTS!E22</f>
         <v>0</v>
       </c>
-      <c r="J23">
+      <c r="J23" s="1">
         <f>IF(H23="",F23,H23)</f>
         <v>0</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="1">
         <f>IF(I23="",G23,I23)</f>
         <v>0</v>
       </c>
@@ -2175,7 +2179,7 @@
       <c r="B26" t="str">
         <v>Sum of Final Low Used</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="1">
         <f>SUM(J15:J23)</f>
         <v>0</v>
       </c>
@@ -2184,7 +2188,7 @@
       <c r="B27" t="str">
         <v>Sum of Final High Used</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="1">
         <f>SUM(K15:K23)</f>
         <v>0</v>
       </c>
@@ -2193,7 +2197,7 @@
       <c r="B28" t="str">
         <v>Base Budget (mid-point)</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="1">
         <f>(C26+C27)/2</f>
         <v>0</v>
       </c>
@@ -2202,7 +2206,7 @@
       <c r="B29" t="str">
         <v>GST (9%)</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="1">
         <f>IF(ASSUMPTIONS!C45,0,ROUND(C28*ASSUMPTIONS!C44,0))</f>
         <v>0</v>
       </c>
@@ -2211,7 +2215,7 @@
       <c r="B30" t="str">
         <v>Contingency</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="1">
         <f>ROUND(C28*INPUTS!C29,0)</f>
         <v>0</v>
       </c>
@@ -2220,7 +2224,7 @@
       <c r="B31" t="str">
         <v>ESTIMATED TOTAL</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="1">
         <f>C28+C29+C30</f>
         <v>0</v>
       </c>
@@ -2516,7 +2520,7 @@
       <c r="B6" t="str">
         <v>Estimated base renovation budget</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <f>INPUTS!F24</f>
         <v>0</v>
       </c>
@@ -2525,7 +2529,7 @@
       <c r="B7" t="str">
         <v>GST (9%)</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <f>INPUTS!F27</f>
         <v>0</v>
       </c>
@@ -2534,7 +2538,7 @@
       <c r="B8" t="str">
         <v>Contingency reserve</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <f>INPUTS!E35</f>
         <v>0</v>
       </c>
@@ -2543,7 +2547,7 @@
       <c r="B9" t="str">
         <v>Optional items subtotal</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <f>INPUTS!E30</f>
         <v>0</v>
       </c>
@@ -2552,7 +2556,7 @@
       <c r="B10" t="str">
         <v>ESTIMATED TOTAL (base + GST + contingency)</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <f>INPUTS!E31</f>
         <v>0</v>
       </c>
@@ -2561,7 +2565,7 @@
       <c r="B11" t="str">
         <v>Renovation loan planned</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <f>INPUTS!C34</f>
         <v>0</v>
       </c>
@@ -2570,7 +2574,7 @@
       <c r="B12" t="str">
         <v>CASH YOU MUST COVER (total − loan)</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <f>INPUTS!E36</f>
         <v>0</v>
       </c>
@@ -2584,7 +2588,7 @@
       <c r="B15" t="str">
         <v>Low planning range</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <f>INPUTS!F25</f>
         <v>0</v>
       </c>
@@ -2593,7 +2597,7 @@
       <c r="B16" t="str">
         <v>High planning range</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <f>INPUTS!F26</f>
         <v>0</v>
       </c>
@@ -2621,11 +2625,11 @@
       <c r="B20" t="str">
         <v>Kitchen renovation</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <f>(INPUTS!F13+INPUTS!G13)/2</f>
         <v>0</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F13+INPUTS!G13)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2638,11 +2642,11 @@
       <c r="B21" t="str">
         <v>Bathroom renovation</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="1">
         <f>(INPUTS!F14+INPUTS!G14)/2</f>
         <v>0</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F14+INPUTS!G14)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2655,11 +2659,11 @@
       <c r="B22" t="str">
         <v>Flooring</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <f>(INPUTS!F15+INPUTS!G15)/2</f>
         <v>0</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F15+INPUTS!G15)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2672,11 +2676,11 @@
       <c r="B23" t="str">
         <v>Painting</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="1">
         <f>(INPUTS!F16+INPUTS!G16)/2</f>
         <v>0</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F16+INPUTS!G16)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2689,11 +2693,11 @@
       <c r="B24" t="str">
         <v>Carpentry</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="1">
         <f>(INPUTS!F17+INPUTS!G17)/2</f>
         <v>0</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F17+INPUTS!G17)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2706,11 +2710,11 @@
       <c r="B25" t="str">
         <v>Electrical</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="1">
         <f>(INPUTS!F18+INPUTS!G18)/2</f>
         <v>0</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F18+INPUTS!G18)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2723,11 +2727,11 @@
       <c r="B26" t="str">
         <v>Hacking</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="1">
         <f>(INPUTS!F19+INPUTS!G19)/2</f>
         <v>0</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F19+INPUTS!G19)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2740,11 +2744,11 @@
       <c r="B27" t="str">
         <v>Built-in furniture</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="1">
         <f>(INPUTS!F20+INPUTS!G20)/2</f>
         <v>0</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F20+INPUTS!G20)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2757,11 +2761,11 @@
       <c r="B28" t="str">
         <v>Appliances / optional items</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="1">
         <f>(INPUTS!F21+INPUTS!G21)/2</f>
         <v>0</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F21+INPUTS!G21)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2774,11 +2778,11 @@
       <c r="B29" t="str">
         <v>User-defined costs</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="1">
         <f>(INPUTS!F22+INPUTS!G22)/2</f>
         <v>0</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="2">
         <f>IF(INPUTS!F24=0,0,((INPUTS!F22+INPUTS!G22)/2)/INPUTS!F24)</f>
         <v>0</v>
       </c>
@@ -2796,7 +2800,7 @@
       <c r="B32" t="str">
         <v>Maximum category amount</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="1">
         <f>MAX(C21:C29)</f>
         <v>0</v>
       </c>
@@ -2820,7 +2824,7 @@
         <f>INPUTS!B40</f>
         <v>0</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="1">
         <f>INPUTS!D40</f>
         <v>0</v>
       </c>
@@ -2834,7 +2838,7 @@
         <f>INPUTS!B41</f>
         <v>0</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="1">
         <f>INPUTS!D41</f>
         <v>0</v>
       </c>
@@ -2848,7 +2852,7 @@
         <f>INPUTS!B42</f>
         <v>0</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="1">
         <f>INPUTS!D42</f>
         <v>0</v>
       </c>
@@ -2862,7 +2866,7 @@
         <f>INPUTS!B43</f>
         <v>0</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="1">
         <f>INPUTS!D43</f>
         <v>0</v>
       </c>
@@ -2876,7 +2880,7 @@
         <f>INPUTS!B44</f>
         <v>0</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="1">
         <f>INPUTS!D44</f>
         <v>0</v>
       </c>
@@ -2889,7 +2893,7 @@
       <c r="B41" t="str">
         <v>Total (verify = 100%)</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="2">
         <f>INPUTS!C45</f>
         <v>0</v>
       </c>

</xml_diff>